<commit_message>
first commit from me
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -1,34 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DOCS\LPU\2627\Session1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bajaj\OneDrive\Desktop\cap776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8837051-77D3-4D36-92D2-5680DDD8E381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D13D99A-DDA6-4CF3-B985-150E824A7A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Daily Log" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -37,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -199,6 +188,27 @@
   </si>
   <si>
     <t>5. GOOD PRACTICE</t>
+  </si>
+  <si>
+    <t>Anmol Bajaj</t>
+  </si>
+  <si>
+    <t>aug-sep</t>
+  </si>
+  <si>
+    <t>CAP-776</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>SATISFIED</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>day was very hectic because managing both studys as well and startup</t>
   </si>
 </sst>
 </file>
@@ -659,186 +669,186 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A39"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="23" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:1" ht="22.8" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="5"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
     </row>
   </sheetData>
@@ -850,7 +860,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N401"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="11" customWidth="1"/>
@@ -863,7 +873,7 @@
     <col min="14" max="14" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>29</v>
       </c>
@@ -881,33 +891,41 @@
       <c r="M1" s="19"/>
       <c r="N1" s="19"/>
     </row>
-    <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="20" t="s">
+        <v>54</v>
+      </c>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="20"/>
+      <c r="F2" s="20">
+        <v>12618856</v>
+      </c>
       <c r="G2" s="20"/>
     </row>
-    <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="20"/>
+      <c r="B3" s="20" t="s">
+        <v>56</v>
+      </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="20"/>
+      <c r="F3" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="G3" s="20"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>34</v>
       </c>
@@ -925,7 +943,7 @@
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
     </row>
-    <row r="5" spans="1:14" ht="42" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>35</v>
       </c>
@@ -969,7 +987,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>46223</v>
       </c>
@@ -1015,29 +1033,53 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
+    <row r="7" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
+        <v>46252</v>
+      </c>
+      <c r="B7" s="14">
+        <v>300</v>
+      </c>
+      <c r="C7" s="14">
+        <v>30</v>
+      </c>
+      <c r="D7" s="14">
+        <v>15</v>
+      </c>
+      <c r="E7" s="14">
+        <v>10</v>
+      </c>
+      <c r="F7" s="14">
+        <v>250</v>
+      </c>
+      <c r="G7" s="14">
+        <v>5</v>
+      </c>
+      <c r="H7" s="14">
+        <v>300</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+        <v>905</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+        <v>535</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -1059,7 +1101,7 @@
       <c r="M8" s="16"/>
       <c r="N8" s="17"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -1081,7 +1123,7 @@
       <c r="M9" s="16"/>
       <c r="N9" s="17"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -1103,7 +1145,7 @@
       <c r="M10" s="16"/>
       <c r="N10" s="17"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -1125,7 +1167,7 @@
       <c r="M11" s="16"/>
       <c r="N11" s="17"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -1147,7 +1189,7 @@
       <c r="M12" s="16"/>
       <c r="N12" s="17"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -1169,7 +1211,7 @@
       <c r="M13" s="16"/>
       <c r="N13" s="17"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -1191,7 +1233,7 @@
       <c r="M14" s="16"/>
       <c r="N14" s="17"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
@@ -1213,7 +1255,7 @@
       <c r="M15" s="16"/>
       <c r="N15" s="17"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
@@ -1235,7 +1277,7 @@
       <c r="M16" s="16"/>
       <c r="N16" s="17"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -1257,7 +1299,7 @@
       <c r="M17" s="16"/>
       <c r="N17" s="17"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
@@ -1279,7 +1321,7 @@
       <c r="M18" s="16"/>
       <c r="N18" s="17"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -1301,7 +1343,7 @@
       <c r="M19" s="16"/>
       <c r="N19" s="17"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="13"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -1323,7 +1365,7 @@
       <c r="M20" s="16"/>
       <c r="N20" s="17"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
@@ -1345,7 +1387,7 @@
       <c r="M21" s="16"/>
       <c r="N21" s="17"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="13"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -1367,7 +1409,7 @@
       <c r="M22" s="16"/>
       <c r="N22" s="17"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
@@ -1389,7 +1431,7 @@
       <c r="M23" s="16"/>
       <c r="N23" s="17"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -1411,7 +1453,7 @@
       <c r="M24" s="16"/>
       <c r="N24" s="17"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -1433,7 +1475,7 @@
       <c r="M25" s="16"/>
       <c r="N25" s="17"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
@@ -1455,7 +1497,7 @@
       <c r="M26" s="16"/>
       <c r="N26" s="17"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
@@ -1477,7 +1519,7 @@
       <c r="M27" s="16"/>
       <c r="N27" s="17"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -1499,7 +1541,7 @@
       <c r="M28" s="16"/>
       <c r="N28" s="17"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
@@ -1521,7 +1563,7 @@
       <c r="M29" s="16"/>
       <c r="N29" s="17"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -1543,7 +1585,7 @@
       <c r="M30" s="16"/>
       <c r="N30" s="17"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -1565,7 +1607,7 @@
       <c r="M31" s="16"/>
       <c r="N31" s="17"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -1587,7 +1629,7 @@
       <c r="M32" s="16"/>
       <c r="N32" s="17"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -1609,7 +1651,7 @@
       <c r="M33" s="16"/>
       <c r="N33" s="17"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -1631,7 +1673,7 @@
       <c r="M34" s="16"/>
       <c r="N34" s="17"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -1653,7 +1695,7 @@
       <c r="M35" s="16"/>
       <c r="N35" s="17"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -1675,7 +1717,7 @@
       <c r="M36" s="16"/>
       <c r="N36" s="17"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
@@ -1697,7 +1739,7 @@
       <c r="M37" s="16"/>
       <c r="N37" s="17"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
@@ -1719,7 +1761,7 @@
       <c r="M38" s="16"/>
       <c r="N38" s="17"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -1741,7 +1783,7 @@
       <c r="M39" s="16"/>
       <c r="N39" s="17"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -1763,7 +1805,7 @@
       <c r="M40" s="16"/>
       <c r="N40" s="17"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
@@ -1785,7 +1827,7 @@
       <c r="M41" s="16"/>
       <c r="N41" s="17"/>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
@@ -1807,7 +1849,7 @@
       <c r="M42" s="16"/>
       <c r="N42" s="17"/>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="13"/>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -1829,7 +1871,7 @@
       <c r="M43" s="16"/>
       <c r="N43" s="17"/>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="13"/>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -1851,7 +1893,7 @@
       <c r="M44" s="16"/>
       <c r="N44" s="17"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="13"/>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
@@ -1873,7 +1915,7 @@
       <c r="M45" s="16"/>
       <c r="N45" s="17"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="13"/>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
@@ -1895,7 +1937,7 @@
       <c r="M46" s="16"/>
       <c r="N46" s="17"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="13"/>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
@@ -1917,7 +1959,7 @@
       <c r="M47" s="16"/>
       <c r="N47" s="17"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="13"/>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
@@ -1939,7 +1981,7 @@
       <c r="M48" s="16"/>
       <c r="N48" s="17"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>
       <c r="B49" s="14"/>
       <c r="C49" s="14"/>
@@ -1961,7 +2003,7 @@
       <c r="M49" s="16"/>
       <c r="N49" s="17"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
@@ -1983,7 +2025,7 @@
       <c r="M50" s="16"/>
       <c r="N50" s="17"/>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>
       <c r="B51" s="14"/>
       <c r="C51" s="14"/>
@@ -2005,7 +2047,7 @@
       <c r="M51" s="16"/>
       <c r="N51" s="17"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
@@ -2027,7 +2069,7 @@
       <c r="M52" s="16"/>
       <c r="N52" s="17"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -2049,7 +2091,7 @@
       <c r="M53" s="16"/>
       <c r="N53" s="17"/>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -2071,7 +2113,7 @@
       <c r="M54" s="16"/>
       <c r="N54" s="17"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -2093,7 +2135,7 @@
       <c r="M55" s="16"/>
       <c r="N55" s="17"/>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="13"/>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -2115,7 +2157,7 @@
       <c r="M56" s="16"/>
       <c r="N56" s="17"/>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="13"/>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -2137,7 +2179,7 @@
       <c r="M57" s="16"/>
       <c r="N57" s="17"/>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="13"/>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -2159,7 +2201,7 @@
       <c r="M58" s="16"/>
       <c r="N58" s="17"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="13"/>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
@@ -2181,7 +2223,7 @@
       <c r="M59" s="16"/>
       <c r="N59" s="17"/>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="13"/>
       <c r="B60" s="14"/>
       <c r="C60" s="14"/>
@@ -2203,7 +2245,7 @@
       <c r="M60" s="16"/>
       <c r="N60" s="17"/>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="13"/>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
@@ -2225,7 +2267,7 @@
       <c r="M61" s="16"/>
       <c r="N61" s="17"/>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="13"/>
       <c r="B62" s="14"/>
       <c r="C62" s="14"/>
@@ -2247,7 +2289,7 @@
       <c r="M62" s="16"/>
       <c r="N62" s="17"/>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="13"/>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -2269,7 +2311,7 @@
       <c r="M63" s="16"/>
       <c r="N63" s="17"/>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
       <c r="B64" s="14"/>
       <c r="C64" s="14"/>
@@ -2291,7 +2333,7 @@
       <c r="M64" s="16"/>
       <c r="N64" s="17"/>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="13"/>
       <c r="B65" s="14"/>
       <c r="C65" s="14"/>
@@ -2313,7 +2355,7 @@
       <c r="M65" s="16"/>
       <c r="N65" s="17"/>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="13"/>
       <c r="B66" s="14"/>
       <c r="C66" s="14"/>
@@ -2335,7 +2377,7 @@
       <c r="M66" s="16"/>
       <c r="N66" s="17"/>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="13"/>
       <c r="B67" s="14"/>
       <c r="C67" s="14"/>
@@ -2357,7 +2399,7 @@
       <c r="M67" s="16"/>
       <c r="N67" s="17"/>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="13"/>
       <c r="B68" s="14"/>
       <c r="C68" s="14"/>
@@ -2379,7 +2421,7 @@
       <c r="M68" s="16"/>
       <c r="N68" s="17"/>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="13"/>
       <c r="B69" s="14"/>
       <c r="C69" s="14"/>
@@ -2401,7 +2443,7 @@
       <c r="M69" s="16"/>
       <c r="N69" s="17"/>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="13"/>
       <c r="B70" s="14"/>
       <c r="C70" s="14"/>
@@ -2423,7 +2465,7 @@
       <c r="M70" s="16"/>
       <c r="N70" s="17"/>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="13"/>
       <c r="B71" s="14"/>
       <c r="C71" s="14"/>
@@ -2445,7 +2487,7 @@
       <c r="M71" s="16"/>
       <c r="N71" s="17"/>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="13"/>
       <c r="B72" s="14"/>
       <c r="C72" s="14"/>
@@ -2467,7 +2509,7 @@
       <c r="M72" s="16"/>
       <c r="N72" s="17"/>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="13"/>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
@@ -2489,7 +2531,7 @@
       <c r="M73" s="16"/>
       <c r="N73" s="17"/>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="13"/>
       <c r="B74" s="14"/>
       <c r="C74" s="14"/>
@@ -2511,7 +2553,7 @@
       <c r="M74" s="16"/>
       <c r="N74" s="17"/>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="13"/>
       <c r="B75" s="14"/>
       <c r="C75" s="14"/>
@@ -2533,7 +2575,7 @@
       <c r="M75" s="16"/>
       <c r="N75" s="17"/>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="13"/>
       <c r="B76" s="14"/>
       <c r="C76" s="14"/>
@@ -2555,7 +2597,7 @@
       <c r="M76" s="16"/>
       <c r="N76" s="17"/>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="13"/>
       <c r="B77" s="14"/>
       <c r="C77" s="14"/>
@@ -2577,7 +2619,7 @@
       <c r="M77" s="16"/>
       <c r="N77" s="17"/>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="13"/>
       <c r="B78" s="14"/>
       <c r="C78" s="14"/>
@@ -2599,7 +2641,7 @@
       <c r="M78" s="16"/>
       <c r="N78" s="17"/>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" s="13"/>
       <c r="B79" s="14"/>
       <c r="C79" s="14"/>
@@ -2621,7 +2663,7 @@
       <c r="M79" s="16"/>
       <c r="N79" s="17"/>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" s="13"/>
       <c r="B80" s="14"/>
       <c r="C80" s="14"/>
@@ -2643,7 +2685,7 @@
       <c r="M80" s="16"/>
       <c r="N80" s="17"/>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="13"/>
       <c r="B81" s="14"/>
       <c r="C81" s="14"/>
@@ -2665,7 +2707,7 @@
       <c r="M81" s="16"/>
       <c r="N81" s="17"/>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="13"/>
       <c r="B82" s="14"/>
       <c r="C82" s="14"/>
@@ -2687,7 +2729,7 @@
       <c r="M82" s="16"/>
       <c r="N82" s="17"/>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="13"/>
       <c r="B83" s="14"/>
       <c r="C83" s="14"/>
@@ -2709,7 +2751,7 @@
       <c r="M83" s="16"/>
       <c r="N83" s="17"/>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" s="13"/>
       <c r="B84" s="14"/>
       <c r="C84" s="14"/>
@@ -2731,7 +2773,7 @@
       <c r="M84" s="16"/>
       <c r="N84" s="17"/>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" s="13"/>
       <c r="B85" s="14"/>
       <c r="C85" s="14"/>
@@ -2753,7 +2795,7 @@
       <c r="M85" s="16"/>
       <c r="N85" s="17"/>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" s="13"/>
       <c r="B86" s="14"/>
       <c r="C86" s="14"/>
@@ -2775,7 +2817,7 @@
       <c r="M86" s="16"/>
       <c r="N86" s="17"/>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" s="13"/>
       <c r="B87" s="14"/>
       <c r="C87" s="14"/>
@@ -2797,7 +2839,7 @@
       <c r="M87" s="16"/>
       <c r="N87" s="17"/>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="13"/>
       <c r="B88" s="14"/>
       <c r="C88" s="14"/>
@@ -2819,7 +2861,7 @@
       <c r="M88" s="16"/>
       <c r="N88" s="17"/>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" s="13"/>
       <c r="B89" s="14"/>
       <c r="C89" s="14"/>
@@ -2841,7 +2883,7 @@
       <c r="M89" s="16"/>
       <c r="N89" s="17"/>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" s="13"/>
       <c r="B90" s="14"/>
       <c r="C90" s="14"/>
@@ -2863,7 +2905,7 @@
       <c r="M90" s="16"/>
       <c r="N90" s="17"/>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" s="13"/>
       <c r="B91" s="14"/>
       <c r="C91" s="14"/>
@@ -2885,7 +2927,7 @@
       <c r="M91" s="16"/>
       <c r="N91" s="17"/>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" s="13"/>
       <c r="B92" s="14"/>
       <c r="C92" s="14"/>
@@ -2907,7 +2949,7 @@
       <c r="M92" s="16"/>
       <c r="N92" s="17"/>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" s="13"/>
       <c r="B93" s="14"/>
       <c r="C93" s="14"/>
@@ -2929,7 +2971,7 @@
       <c r="M93" s="16"/>
       <c r="N93" s="17"/>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" s="13"/>
       <c r="B94" s="14"/>
       <c r="C94" s="14"/>
@@ -2951,7 +2993,7 @@
       <c r="M94" s="16"/>
       <c r="N94" s="17"/>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="13"/>
       <c r="B95" s="14"/>
       <c r="C95" s="14"/>
@@ -2973,7 +3015,7 @@
       <c r="M95" s="16"/>
       <c r="N95" s="17"/>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" s="13"/>
       <c r="B96" s="14"/>
       <c r="C96" s="14"/>
@@ -2995,7 +3037,7 @@
       <c r="M96" s="16"/>
       <c r="N96" s="17"/>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" s="13"/>
       <c r="B97" s="14"/>
       <c r="C97" s="14"/>
@@ -3017,7 +3059,7 @@
       <c r="M97" s="16"/>
       <c r="N97" s="17"/>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" s="13"/>
       <c r="B98" s="14"/>
       <c r="C98" s="14"/>
@@ -3039,7 +3081,7 @@
       <c r="M98" s="16"/>
       <c r="N98" s="17"/>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" s="13"/>
       <c r="B99" s="14"/>
       <c r="C99" s="14"/>
@@ -3061,7 +3103,7 @@
       <c r="M99" s="16"/>
       <c r="N99" s="17"/>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" s="13"/>
       <c r="B100" s="14"/>
       <c r="C100" s="14"/>
@@ -3083,7 +3125,7 @@
       <c r="M100" s="16"/>
       <c r="N100" s="17"/>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" s="13"/>
       <c r="B101" s="14"/>
       <c r="C101" s="14"/>
@@ -3105,7 +3147,7 @@
       <c r="M101" s="16"/>
       <c r="N101" s="17"/>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="13"/>
       <c r="B102" s="14"/>
       <c r="C102" s="14"/>
@@ -3127,7 +3169,7 @@
       <c r="M102" s="16"/>
       <c r="N102" s="17"/>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A103" s="13"/>
       <c r="B103" s="14"/>
       <c r="C103" s="14"/>
@@ -3149,7 +3191,7 @@
       <c r="M103" s="16"/>
       <c r="N103" s="17"/>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" s="13"/>
       <c r="B104" s="14"/>
       <c r="C104" s="14"/>
@@ -3171,7 +3213,7 @@
       <c r="M104" s="16"/>
       <c r="N104" s="17"/>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A105" s="13"/>
       <c r="B105" s="14"/>
       <c r="C105" s="14"/>
@@ -3193,7 +3235,7 @@
       <c r="M105" s="16"/>
       <c r="N105" s="17"/>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A106" s="13"/>
       <c r="B106" s="14"/>
       <c r="C106" s="14"/>
@@ -3215,7 +3257,7 @@
       <c r="M106" s="16"/>
       <c r="N106" s="17"/>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" s="13"/>
       <c r="B107" s="14"/>
       <c r="C107" s="14"/>
@@ -3237,7 +3279,7 @@
       <c r="M107" s="16"/>
       <c r="N107" s="17"/>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" s="13"/>
       <c r="B108" s="14"/>
       <c r="C108" s="14"/>
@@ -3259,7 +3301,7 @@
       <c r="M108" s="16"/>
       <c r="N108" s="17"/>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" s="13"/>
       <c r="B109" s="14"/>
       <c r="C109" s="14"/>
@@ -3281,7 +3323,7 @@
       <c r="M109" s="16"/>
       <c r="N109" s="17"/>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" s="13"/>
       <c r="B110" s="14"/>
       <c r="C110" s="14"/>
@@ -3303,7 +3345,7 @@
       <c r="M110" s="16"/>
       <c r="N110" s="17"/>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A111" s="13"/>
       <c r="B111" s="14"/>
       <c r="C111" s="14"/>
@@ -3325,7 +3367,7 @@
       <c r="M111" s="16"/>
       <c r="N111" s="17"/>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A112" s="13"/>
       <c r="B112" s="14"/>
       <c r="C112" s="14"/>
@@ -3347,7 +3389,7 @@
       <c r="M112" s="16"/>
       <c r="N112" s="17"/>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A113" s="13"/>
       <c r="B113" s="14"/>
       <c r="C113" s="14"/>
@@ -3369,7 +3411,7 @@
       <c r="M113" s="16"/>
       <c r="N113" s="17"/>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" s="13"/>
       <c r="B114" s="14"/>
       <c r="C114" s="14"/>
@@ -3391,7 +3433,7 @@
       <c r="M114" s="16"/>
       <c r="N114" s="17"/>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A115" s="13"/>
       <c r="B115" s="14"/>
       <c r="C115" s="14"/>
@@ -3413,7 +3455,7 @@
       <c r="M115" s="16"/>
       <c r="N115" s="17"/>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" s="13"/>
       <c r="B116" s="14"/>
       <c r="C116" s="14"/>
@@ -3435,7 +3477,7 @@
       <c r="M116" s="16"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A117" s="13"/>
       <c r="B117" s="14"/>
       <c r="C117" s="14"/>
@@ -3457,7 +3499,7 @@
       <c r="M117" s="16"/>
       <c r="N117" s="17"/>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A118" s="13"/>
       <c r="B118" s="14"/>
       <c r="C118" s="14"/>
@@ -3479,7 +3521,7 @@
       <c r="M118" s="16"/>
       <c r="N118" s="17"/>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A119" s="13"/>
       <c r="B119" s="14"/>
       <c r="C119" s="14"/>
@@ -3501,7 +3543,7 @@
       <c r="M119" s="16"/>
       <c r="N119" s="17"/>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A120" s="13"/>
       <c r="B120" s="14"/>
       <c r="C120" s="14"/>
@@ -3523,7 +3565,7 @@
       <c r="M120" s="16"/>
       <c r="N120" s="17"/>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A121" s="13"/>
       <c r="B121" s="14"/>
       <c r="C121" s="14"/>
@@ -3545,7 +3587,7 @@
       <c r="M121" s="16"/>
       <c r="N121" s="17"/>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A122" s="13"/>
       <c r="B122" s="14"/>
       <c r="C122" s="14"/>
@@ -3567,7 +3609,7 @@
       <c r="M122" s="16"/>
       <c r="N122" s="17"/>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A123" s="13"/>
       <c r="B123" s="14"/>
       <c r="C123" s="14"/>
@@ -3589,7 +3631,7 @@
       <c r="M123" s="16"/>
       <c r="N123" s="17"/>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A124" s="13"/>
       <c r="B124" s="14"/>
       <c r="C124" s="14"/>
@@ -3611,7 +3653,7 @@
       <c r="M124" s="16"/>
       <c r="N124" s="17"/>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" s="13"/>
       <c r="B125" s="14"/>
       <c r="C125" s="14"/>
@@ -3633,7 +3675,7 @@
       <c r="M125" s="16"/>
       <c r="N125" s="17"/>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A126" s="13"/>
       <c r="B126" s="14"/>
       <c r="C126" s="14"/>
@@ -3655,7 +3697,7 @@
       <c r="M126" s="16"/>
       <c r="N126" s="17"/>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A127" s="13"/>
       <c r="B127" s="14"/>
       <c r="C127" s="14"/>
@@ -3677,7 +3719,7 @@
       <c r="M127" s="16"/>
       <c r="N127" s="17"/>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A128" s="13"/>
       <c r="B128" s="14"/>
       <c r="C128" s="14"/>
@@ -3699,7 +3741,7 @@
       <c r="M128" s="16"/>
       <c r="N128" s="17"/>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A129" s="13"/>
       <c r="B129" s="14"/>
       <c r="C129" s="14"/>
@@ -3721,7 +3763,7 @@
       <c r="M129" s="16"/>
       <c r="N129" s="17"/>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A130" s="13"/>
       <c r="B130" s="14"/>
       <c r="C130" s="14"/>
@@ -3743,7 +3785,7 @@
       <c r="M130" s="16"/>
       <c r="N130" s="17"/>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A131" s="13"/>
       <c r="B131" s="14"/>
       <c r="C131" s="14"/>
@@ -3765,7 +3807,7 @@
       <c r="M131" s="16"/>
       <c r="N131" s="17"/>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A132" s="13"/>
       <c r="B132" s="14"/>
       <c r="C132" s="14"/>
@@ -3787,7 +3829,7 @@
       <c r="M132" s="16"/>
       <c r="N132" s="17"/>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A133" s="13"/>
       <c r="B133" s="14"/>
       <c r="C133" s="14"/>
@@ -3809,7 +3851,7 @@
       <c r="M133" s="16"/>
       <c r="N133" s="17"/>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A134" s="13"/>
       <c r="B134" s="14"/>
       <c r="C134" s="14"/>
@@ -3831,7 +3873,7 @@
       <c r="M134" s="16"/>
       <c r="N134" s="17"/>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A135" s="13"/>
       <c r="B135" s="14"/>
       <c r="C135" s="14"/>
@@ -3853,7 +3895,7 @@
       <c r="M135" s="16"/>
       <c r="N135" s="17"/>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A136" s="13"/>
       <c r="B136" s="14"/>
       <c r="C136" s="14"/>
@@ -3875,7 +3917,7 @@
       <c r="M136" s="16"/>
       <c r="N136" s="17"/>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A137" s="13"/>
       <c r="B137" s="14"/>
       <c r="C137" s="14"/>
@@ -3897,7 +3939,7 @@
       <c r="M137" s="16"/>
       <c r="N137" s="17"/>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A138" s="13"/>
       <c r="B138" s="14"/>
       <c r="C138" s="14"/>
@@ -3919,7 +3961,7 @@
       <c r="M138" s="16"/>
       <c r="N138" s="17"/>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139" s="13"/>
       <c r="B139" s="14"/>
       <c r="C139" s="14"/>
@@ -3941,7 +3983,7 @@
       <c r="M139" s="16"/>
       <c r="N139" s="17"/>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140" s="13"/>
       <c r="B140" s="14"/>
       <c r="C140" s="14"/>
@@ -3963,7 +4005,7 @@
       <c r="M140" s="16"/>
       <c r="N140" s="17"/>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141" s="13"/>
       <c r="B141" s="14"/>
       <c r="C141" s="14"/>
@@ -3985,7 +4027,7 @@
       <c r="M141" s="16"/>
       <c r="N141" s="17"/>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142" s="13"/>
       <c r="B142" s="14"/>
       <c r="C142" s="14"/>
@@ -4007,7 +4049,7 @@
       <c r="M142" s="16"/>
       <c r="N142" s="17"/>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143" s="13"/>
       <c r="B143" s="14"/>
       <c r="C143" s="14"/>
@@ -4029,7 +4071,7 @@
       <c r="M143" s="16"/>
       <c r="N143" s="17"/>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144" s="13"/>
       <c r="B144" s="14"/>
       <c r="C144" s="14"/>
@@ -4051,7 +4093,7 @@
       <c r="M144" s="16"/>
       <c r="N144" s="17"/>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A145" s="13"/>
       <c r="B145" s="14"/>
       <c r="C145" s="14"/>
@@ -4073,7 +4115,7 @@
       <c r="M145" s="16"/>
       <c r="N145" s="17"/>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A146" s="13"/>
       <c r="B146" s="14"/>
       <c r="C146" s="14"/>
@@ -4095,7 +4137,7 @@
       <c r="M146" s="16"/>
       <c r="N146" s="17"/>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" s="13"/>
       <c r="B147" s="14"/>
       <c r="C147" s="14"/>
@@ -4117,7 +4159,7 @@
       <c r="M147" s="16"/>
       <c r="N147" s="17"/>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" s="13"/>
       <c r="B148" s="14"/>
       <c r="C148" s="14"/>
@@ -4139,7 +4181,7 @@
       <c r="M148" s="16"/>
       <c r="N148" s="17"/>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" s="13"/>
       <c r="B149" s="14"/>
       <c r="C149" s="14"/>
@@ -4161,7 +4203,7 @@
       <c r="M149" s="16"/>
       <c r="N149" s="17"/>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" s="13"/>
       <c r="B150" s="14"/>
       <c r="C150" s="14"/>
@@ -4183,7 +4225,7 @@
       <c r="M150" s="16"/>
       <c r="N150" s="17"/>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" s="13"/>
       <c r="B151" s="14"/>
       <c r="C151" s="14"/>
@@ -4205,7 +4247,7 @@
       <c r="M151" s="16"/>
       <c r="N151" s="17"/>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" s="13"/>
       <c r="B152" s="14"/>
       <c r="C152" s="14"/>
@@ -4227,7 +4269,7 @@
       <c r="M152" s="16"/>
       <c r="N152" s="17"/>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" s="13"/>
       <c r="B153" s="14"/>
       <c r="C153" s="14"/>
@@ -4249,7 +4291,7 @@
       <c r="M153" s="16"/>
       <c r="N153" s="17"/>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" s="13"/>
       <c r="B154" s="14"/>
       <c r="C154" s="14"/>
@@ -4271,7 +4313,7 @@
       <c r="M154" s="16"/>
       <c r="N154" s="17"/>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" s="13"/>
       <c r="B155" s="14"/>
       <c r="C155" s="14"/>
@@ -4293,7 +4335,7 @@
       <c r="M155" s="16"/>
       <c r="N155" s="17"/>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A156" s="13"/>
       <c r="B156" s="14"/>
       <c r="C156" s="14"/>
@@ -4315,7 +4357,7 @@
       <c r="M156" s="16"/>
       <c r="N156" s="17"/>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A157" s="13"/>
       <c r="B157" s="14"/>
       <c r="C157" s="14"/>
@@ -4337,7 +4379,7 @@
       <c r="M157" s="16"/>
       <c r="N157" s="17"/>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A158" s="13"/>
       <c r="B158" s="14"/>
       <c r="C158" s="14"/>
@@ -4359,7 +4401,7 @@
       <c r="M158" s="16"/>
       <c r="N158" s="17"/>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A159" s="13"/>
       <c r="B159" s="14"/>
       <c r="C159" s="14"/>
@@ -4381,7 +4423,7 @@
       <c r="M159" s="16"/>
       <c r="N159" s="17"/>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A160" s="13"/>
       <c r="B160" s="14"/>
       <c r="C160" s="14"/>
@@ -4403,7 +4445,7 @@
       <c r="M160" s="16"/>
       <c r="N160" s="17"/>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A161" s="13"/>
       <c r="B161" s="14"/>
       <c r="C161" s="14"/>
@@ -4425,7 +4467,7 @@
       <c r="M161" s="16"/>
       <c r="N161" s="17"/>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A162" s="13"/>
       <c r="B162" s="14"/>
       <c r="C162" s="14"/>
@@ -4447,7 +4489,7 @@
       <c r="M162" s="16"/>
       <c r="N162" s="17"/>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A163" s="13"/>
       <c r="B163" s="14"/>
       <c r="C163" s="14"/>
@@ -4469,7 +4511,7 @@
       <c r="M163" s="16"/>
       <c r="N163" s="17"/>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A164" s="13"/>
       <c r="B164" s="14"/>
       <c r="C164" s="14"/>
@@ -4491,7 +4533,7 @@
       <c r="M164" s="16"/>
       <c r="N164" s="17"/>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A165" s="13"/>
       <c r="B165" s="14"/>
       <c r="C165" s="14"/>
@@ -4513,7 +4555,7 @@
       <c r="M165" s="16"/>
       <c r="N165" s="17"/>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A166" s="13"/>
       <c r="B166" s="14"/>
       <c r="C166" s="14"/>
@@ -4535,7 +4577,7 @@
       <c r="M166" s="16"/>
       <c r="N166" s="17"/>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A167" s="13"/>
       <c r="B167" s="14"/>
       <c r="C167" s="14"/>
@@ -4557,7 +4599,7 @@
       <c r="M167" s="16"/>
       <c r="N167" s="17"/>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A168" s="13"/>
       <c r="B168" s="14"/>
       <c r="C168" s="14"/>
@@ -4579,7 +4621,7 @@
       <c r="M168" s="16"/>
       <c r="N168" s="17"/>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A169" s="13"/>
       <c r="B169" s="14"/>
       <c r="C169" s="14"/>
@@ -4601,7 +4643,7 @@
       <c r="M169" s="16"/>
       <c r="N169" s="17"/>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A170" s="13"/>
       <c r="B170" s="14"/>
       <c r="C170" s="14"/>
@@ -4623,7 +4665,7 @@
       <c r="M170" s="16"/>
       <c r="N170" s="17"/>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A171" s="13"/>
       <c r="B171" s="14"/>
       <c r="C171" s="14"/>
@@ -4645,7 +4687,7 @@
       <c r="M171" s="16"/>
       <c r="N171" s="17"/>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A172" s="13"/>
       <c r="B172" s="14"/>
       <c r="C172" s="14"/>
@@ -4667,7 +4709,7 @@
       <c r="M172" s="16"/>
       <c r="N172" s="17"/>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A173" s="13"/>
       <c r="B173" s="14"/>
       <c r="C173" s="14"/>
@@ -4689,7 +4731,7 @@
       <c r="M173" s="16"/>
       <c r="N173" s="17"/>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A174" s="13"/>
       <c r="B174" s="14"/>
       <c r="C174" s="14"/>
@@ -4711,7 +4753,7 @@
       <c r="M174" s="16"/>
       <c r="N174" s="17"/>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A175" s="13"/>
       <c r="B175" s="14"/>
       <c r="C175" s="14"/>
@@ -4733,7 +4775,7 @@
       <c r="M175" s="16"/>
       <c r="N175" s="17"/>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A176" s="13"/>
       <c r="B176" s="14"/>
       <c r="C176" s="14"/>
@@ -4755,7 +4797,7 @@
       <c r="M176" s="16"/>
       <c r="N176" s="17"/>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A177" s="13"/>
       <c r="B177" s="14"/>
       <c r="C177" s="14"/>
@@ -4777,7 +4819,7 @@
       <c r="M177" s="16"/>
       <c r="N177" s="17"/>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A178" s="13"/>
       <c r="B178" s="14"/>
       <c r="C178" s="14"/>
@@ -4799,7 +4841,7 @@
       <c r="M178" s="16"/>
       <c r="N178" s="17"/>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A179" s="13"/>
       <c r="B179" s="14"/>
       <c r="C179" s="14"/>
@@ -4821,7 +4863,7 @@
       <c r="M179" s="16"/>
       <c r="N179" s="17"/>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A180" s="13"/>
       <c r="B180" s="14"/>
       <c r="C180" s="14"/>
@@ -4843,7 +4885,7 @@
       <c r="M180" s="16"/>
       <c r="N180" s="17"/>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A181" s="13"/>
       <c r="B181" s="14"/>
       <c r="C181" s="14"/>
@@ -4865,7 +4907,7 @@
       <c r="M181" s="16"/>
       <c r="N181" s="17"/>
     </row>
-    <row r="182" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A182" s="13"/>
       <c r="B182" s="14"/>
       <c r="C182" s="14"/>
@@ -4887,7 +4929,7 @@
       <c r="M182" s="16"/>
       <c r="N182" s="17"/>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A183" s="13"/>
       <c r="B183" s="14"/>
       <c r="C183" s="14"/>
@@ -4909,7 +4951,7 @@
       <c r="M183" s="16"/>
       <c r="N183" s="17"/>
     </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A184" s="13"/>
       <c r="B184" s="14"/>
       <c r="C184" s="14"/>
@@ -4931,7 +4973,7 @@
       <c r="M184" s="16"/>
       <c r="N184" s="17"/>
     </row>
-    <row r="185" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A185" s="13"/>
       <c r="B185" s="14"/>
       <c r="C185" s="14"/>
@@ -4953,7 +4995,7 @@
       <c r="M185" s="16"/>
       <c r="N185" s="17"/>
     </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A186" s="13"/>
       <c r="B186" s="14"/>
       <c r="C186" s="14"/>
@@ -4975,7 +5017,7 @@
       <c r="M186" s="16"/>
       <c r="N186" s="17"/>
     </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A187" s="13"/>
       <c r="B187" s="14"/>
       <c r="C187" s="14"/>
@@ -4997,7 +5039,7 @@
       <c r="M187" s="16"/>
       <c r="N187" s="17"/>
     </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A188" s="13"/>
       <c r="B188" s="14"/>
       <c r="C188" s="14"/>
@@ -5019,7 +5061,7 @@
       <c r="M188" s="16"/>
       <c r="N188" s="17"/>
     </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A189" s="13"/>
       <c r="B189" s="14"/>
       <c r="C189" s="14"/>
@@ -5041,7 +5083,7 @@
       <c r="M189" s="16"/>
       <c r="N189" s="17"/>
     </row>
-    <row r="190" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A190" s="13"/>
       <c r="B190" s="14"/>
       <c r="C190" s="14"/>
@@ -5063,7 +5105,7 @@
       <c r="M190" s="16"/>
       <c r="N190" s="17"/>
     </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A191" s="13"/>
       <c r="B191" s="14"/>
       <c r="C191" s="14"/>
@@ -5085,7 +5127,7 @@
       <c r="M191" s="16"/>
       <c r="N191" s="17"/>
     </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A192" s="13"/>
       <c r="B192" s="14"/>
       <c r="C192" s="14"/>
@@ -5107,7 +5149,7 @@
       <c r="M192" s="16"/>
       <c r="N192" s="17"/>
     </row>
-    <row r="193" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A193" s="13"/>
       <c r="B193" s="14"/>
       <c r="C193" s="14"/>
@@ -5129,7 +5171,7 @@
       <c r="M193" s="16"/>
       <c r="N193" s="17"/>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A194" s="13"/>
       <c r="B194" s="14"/>
       <c r="C194" s="14"/>
@@ -5151,7 +5193,7 @@
       <c r="M194" s="16"/>
       <c r="N194" s="17"/>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A195" s="13"/>
       <c r="B195" s="14"/>
       <c r="C195" s="14"/>
@@ -5173,7 +5215,7 @@
       <c r="M195" s="16"/>
       <c r="N195" s="17"/>
     </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A196" s="13"/>
       <c r="B196" s="14"/>
       <c r="C196" s="14"/>
@@ -5195,7 +5237,7 @@
       <c r="M196" s="16"/>
       <c r="N196" s="17"/>
     </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A197" s="13"/>
       <c r="B197" s="14"/>
       <c r="C197" s="14"/>
@@ -5217,7 +5259,7 @@
       <c r="M197" s="16"/>
       <c r="N197" s="17"/>
     </row>
-    <row r="198" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A198" s="13"/>
       <c r="B198" s="14"/>
       <c r="C198" s="14"/>
@@ -5239,7 +5281,7 @@
       <c r="M198" s="16"/>
       <c r="N198" s="17"/>
     </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A199" s="13"/>
       <c r="B199" s="14"/>
       <c r="C199" s="14"/>
@@ -5261,7 +5303,7 @@
       <c r="M199" s="16"/>
       <c r="N199" s="17"/>
     </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A200" s="13"/>
       <c r="B200" s="14"/>
       <c r="C200" s="14"/>
@@ -5283,7 +5325,7 @@
       <c r="M200" s="16"/>
       <c r="N200" s="17"/>
     </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A201" s="13"/>
       <c r="B201" s="14"/>
       <c r="C201" s="14"/>
@@ -5305,7 +5347,7 @@
       <c r="M201" s="16"/>
       <c r="N201" s="17"/>
     </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A202" s="13"/>
       <c r="B202" s="14"/>
       <c r="C202" s="14"/>
@@ -5327,7 +5369,7 @@
       <c r="M202" s="16"/>
       <c r="N202" s="17"/>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A203" s="13"/>
       <c r="B203" s="14"/>
       <c r="C203" s="14"/>
@@ -5349,7 +5391,7 @@
       <c r="M203" s="16"/>
       <c r="N203" s="17"/>
     </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A204" s="13"/>
       <c r="B204" s="14"/>
       <c r="C204" s="14"/>
@@ -5371,7 +5413,7 @@
       <c r="M204" s="16"/>
       <c r="N204" s="17"/>
     </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A205" s="13"/>
       <c r="B205" s="14"/>
       <c r="C205" s="14"/>
@@ -5393,7 +5435,7 @@
       <c r="M205" s="16"/>
       <c r="N205" s="17"/>
     </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A206" s="13"/>
       <c r="B206" s="14"/>
       <c r="C206" s="14"/>
@@ -5415,7 +5457,7 @@
       <c r="M206" s="16"/>
       <c r="N206" s="17"/>
     </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A207" s="13"/>
       <c r="B207" s="14"/>
       <c r="C207" s="14"/>
@@ -5437,7 +5479,7 @@
       <c r="M207" s="16"/>
       <c r="N207" s="17"/>
     </row>
-    <row r="208" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A208" s="13"/>
       <c r="B208" s="14"/>
       <c r="C208" s="14"/>
@@ -5459,7 +5501,7 @@
       <c r="M208" s="16"/>
       <c r="N208" s="17"/>
     </row>
-    <row r="209" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A209" s="13"/>
       <c r="B209" s="14"/>
       <c r="C209" s="14"/>
@@ -5481,7 +5523,7 @@
       <c r="M209" s="16"/>
       <c r="N209" s="17"/>
     </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A210" s="13"/>
       <c r="B210" s="14"/>
       <c r="C210" s="14"/>
@@ -5503,7 +5545,7 @@
       <c r="M210" s="16"/>
       <c r="N210" s="17"/>
     </row>
-    <row r="211" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A211" s="13"/>
       <c r="B211" s="14"/>
       <c r="C211" s="14"/>
@@ -5525,7 +5567,7 @@
       <c r="M211" s="16"/>
       <c r="N211" s="17"/>
     </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A212" s="13"/>
       <c r="B212" s="14"/>
       <c r="C212" s="14"/>
@@ -5547,7 +5589,7 @@
       <c r="M212" s="16"/>
       <c r="N212" s="17"/>
     </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A213" s="13"/>
       <c r="B213" s="14"/>
       <c r="C213" s="14"/>
@@ -5569,7 +5611,7 @@
       <c r="M213" s="16"/>
       <c r="N213" s="17"/>
     </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A214" s="13"/>
       <c r="B214" s="14"/>
       <c r="C214" s="14"/>
@@ -5591,7 +5633,7 @@
       <c r="M214" s="16"/>
       <c r="N214" s="17"/>
     </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A215" s="13"/>
       <c r="B215" s="14"/>
       <c r="C215" s="14"/>
@@ -5613,7 +5655,7 @@
       <c r="M215" s="16"/>
       <c r="N215" s="17"/>
     </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A216" s="13"/>
       <c r="B216" s="14"/>
       <c r="C216" s="14"/>
@@ -5635,7 +5677,7 @@
       <c r="M216" s="16"/>
       <c r="N216" s="17"/>
     </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A217" s="13"/>
       <c r="B217" s="14"/>
       <c r="C217" s="14"/>
@@ -5657,7 +5699,7 @@
       <c r="M217" s="16"/>
       <c r="N217" s="17"/>
     </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A218" s="13"/>
       <c r="B218" s="14"/>
       <c r="C218" s="14"/>
@@ -5679,7 +5721,7 @@
       <c r="M218" s="16"/>
       <c r="N218" s="17"/>
     </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A219" s="13"/>
       <c r="B219" s="14"/>
       <c r="C219" s="14"/>
@@ -5701,7 +5743,7 @@
       <c r="M219" s="16"/>
       <c r="N219" s="17"/>
     </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A220" s="13"/>
       <c r="B220" s="14"/>
       <c r="C220" s="14"/>
@@ -5723,7 +5765,7 @@
       <c r="M220" s="16"/>
       <c r="N220" s="17"/>
     </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A221" s="13"/>
       <c r="B221" s="14"/>
       <c r="C221" s="14"/>
@@ -5745,7 +5787,7 @@
       <c r="M221" s="16"/>
       <c r="N221" s="17"/>
     </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A222" s="13"/>
       <c r="B222" s="14"/>
       <c r="C222" s="14"/>
@@ -5767,7 +5809,7 @@
       <c r="M222" s="16"/>
       <c r="N222" s="17"/>
     </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A223" s="13"/>
       <c r="B223" s="14"/>
       <c r="C223" s="14"/>
@@ -5789,7 +5831,7 @@
       <c r="M223" s="16"/>
       <c r="N223" s="17"/>
     </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A224" s="13"/>
       <c r="B224" s="14"/>
       <c r="C224" s="14"/>
@@ -5811,7 +5853,7 @@
       <c r="M224" s="16"/>
       <c r="N224" s="17"/>
     </row>
-    <row r="225" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A225" s="13"/>
       <c r="B225" s="14"/>
       <c r="C225" s="14"/>
@@ -5833,7 +5875,7 @@
       <c r="M225" s="16"/>
       <c r="N225" s="17"/>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A226" s="13"/>
       <c r="B226" s="14"/>
       <c r="C226" s="14"/>
@@ -5855,7 +5897,7 @@
       <c r="M226" s="16"/>
       <c r="N226" s="17"/>
     </row>
-    <row r="227" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A227" s="13"/>
       <c r="B227" s="14"/>
       <c r="C227" s="14"/>
@@ -5877,7 +5919,7 @@
       <c r="M227" s="16"/>
       <c r="N227" s="17"/>
     </row>
-    <row r="228" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A228" s="13"/>
       <c r="B228" s="14"/>
       <c r="C228" s="14"/>
@@ -5899,7 +5941,7 @@
       <c r="M228" s="16"/>
       <c r="N228" s="17"/>
     </row>
-    <row r="229" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A229" s="13"/>
       <c r="B229" s="14"/>
       <c r="C229" s="14"/>
@@ -5921,7 +5963,7 @@
       <c r="M229" s="16"/>
       <c r="N229" s="17"/>
     </row>
-    <row r="230" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A230" s="13"/>
       <c r="B230" s="14"/>
       <c r="C230" s="14"/>
@@ -5943,7 +5985,7 @@
       <c r="M230" s="16"/>
       <c r="N230" s="17"/>
     </row>
-    <row r="231" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A231" s="13"/>
       <c r="B231" s="14"/>
       <c r="C231" s="14"/>
@@ -5965,7 +6007,7 @@
       <c r="M231" s="16"/>
       <c r="N231" s="17"/>
     </row>
-    <row r="232" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A232" s="13"/>
       <c r="B232" s="14"/>
       <c r="C232" s="14"/>
@@ -5987,7 +6029,7 @@
       <c r="M232" s="16"/>
       <c r="N232" s="17"/>
     </row>
-    <row r="233" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A233" s="13"/>
       <c r="B233" s="14"/>
       <c r="C233" s="14"/>
@@ -6009,7 +6051,7 @@
       <c r="M233" s="16"/>
       <c r="N233" s="17"/>
     </row>
-    <row r="234" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A234" s="13"/>
       <c r="B234" s="14"/>
       <c r="C234" s="14"/>
@@ -6031,7 +6073,7 @@
       <c r="M234" s="16"/>
       <c r="N234" s="17"/>
     </row>
-    <row r="235" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A235" s="13"/>
       <c r="B235" s="14"/>
       <c r="C235" s="14"/>
@@ -6053,7 +6095,7 @@
       <c r="M235" s="16"/>
       <c r="N235" s="17"/>
     </row>
-    <row r="236" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A236" s="13"/>
       <c r="B236" s="14"/>
       <c r="C236" s="14"/>
@@ -6075,7 +6117,7 @@
       <c r="M236" s="16"/>
       <c r="N236" s="17"/>
     </row>
-    <row r="237" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A237" s="13"/>
       <c r="B237" s="14"/>
       <c r="C237" s="14"/>
@@ -6097,7 +6139,7 @@
       <c r="M237" s="16"/>
       <c r="N237" s="17"/>
     </row>
-    <row r="238" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A238" s="13"/>
       <c r="B238" s="14"/>
       <c r="C238" s="14"/>
@@ -6119,7 +6161,7 @@
       <c r="M238" s="16"/>
       <c r="N238" s="17"/>
     </row>
-    <row r="239" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A239" s="13"/>
       <c r="B239" s="14"/>
       <c r="C239" s="14"/>
@@ -6141,7 +6183,7 @@
       <c r="M239" s="16"/>
       <c r="N239" s="17"/>
     </row>
-    <row r="240" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A240" s="13"/>
       <c r="B240" s="14"/>
       <c r="C240" s="14"/>
@@ -6163,7 +6205,7 @@
       <c r="M240" s="16"/>
       <c r="N240" s="17"/>
     </row>
-    <row r="241" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A241" s="13"/>
       <c r="B241" s="14"/>
       <c r="C241" s="14"/>
@@ -6185,7 +6227,7 @@
       <c r="M241" s="16"/>
       <c r="N241" s="17"/>
     </row>
-    <row r="242" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A242" s="13"/>
       <c r="B242" s="14"/>
       <c r="C242" s="14"/>
@@ -6207,7 +6249,7 @@
       <c r="M242" s="16"/>
       <c r="N242" s="17"/>
     </row>
-    <row r="243" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A243" s="13"/>
       <c r="B243" s="14"/>
       <c r="C243" s="14"/>
@@ -6229,7 +6271,7 @@
       <c r="M243" s="16"/>
       <c r="N243" s="17"/>
     </row>
-    <row r="244" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A244" s="13"/>
       <c r="B244" s="14"/>
       <c r="C244" s="14"/>
@@ -6251,7 +6293,7 @@
       <c r="M244" s="16"/>
       <c r="N244" s="17"/>
     </row>
-    <row r="245" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A245" s="13"/>
       <c r="B245" s="14"/>
       <c r="C245" s="14"/>
@@ -6273,7 +6315,7 @@
       <c r="M245" s="16"/>
       <c r="N245" s="17"/>
     </row>
-    <row r="246" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A246" s="13"/>
       <c r="B246" s="14"/>
       <c r="C246" s="14"/>
@@ -6295,7 +6337,7 @@
       <c r="M246" s="16"/>
       <c r="N246" s="17"/>
     </row>
-    <row r="247" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A247" s="13"/>
       <c r="B247" s="14"/>
       <c r="C247" s="14"/>
@@ -6317,7 +6359,7 @@
       <c r="M247" s="16"/>
       <c r="N247" s="17"/>
     </row>
-    <row r="248" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A248" s="13"/>
       <c r="B248" s="14"/>
       <c r="C248" s="14"/>
@@ -6339,7 +6381,7 @@
       <c r="M248" s="16"/>
       <c r="N248" s="17"/>
     </row>
-    <row r="249" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A249" s="13"/>
       <c r="B249" s="14"/>
       <c r="C249" s="14"/>
@@ -6361,7 +6403,7 @@
       <c r="M249" s="16"/>
       <c r="N249" s="17"/>
     </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A250" s="13"/>
       <c r="B250" s="14"/>
       <c r="C250" s="14"/>
@@ -6383,7 +6425,7 @@
       <c r="M250" s="16"/>
       <c r="N250" s="17"/>
     </row>
-    <row r="251" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A251" s="13"/>
       <c r="B251" s="14"/>
       <c r="C251" s="14"/>
@@ -6405,7 +6447,7 @@
       <c r="M251" s="16"/>
       <c r="N251" s="17"/>
     </row>
-    <row r="252" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A252" s="13"/>
       <c r="B252" s="14"/>
       <c r="C252" s="14"/>
@@ -6427,7 +6469,7 @@
       <c r="M252" s="16"/>
       <c r="N252" s="17"/>
     </row>
-    <row r="253" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A253" s="13"/>
       <c r="B253" s="14"/>
       <c r="C253" s="14"/>
@@ -6449,7 +6491,7 @@
       <c r="M253" s="16"/>
       <c r="N253" s="17"/>
     </row>
-    <row r="254" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A254" s="13"/>
       <c r="B254" s="14"/>
       <c r="C254" s="14"/>
@@ -6471,7 +6513,7 @@
       <c r="M254" s="16"/>
       <c r="N254" s="17"/>
     </row>
-    <row r="255" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A255" s="13"/>
       <c r="B255" s="14"/>
       <c r="C255" s="14"/>
@@ -6493,7 +6535,7 @@
       <c r="M255" s="16"/>
       <c r="N255" s="17"/>
     </row>
-    <row r="256" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A256" s="13"/>
       <c r="B256" s="14"/>
       <c r="C256" s="14"/>
@@ -6515,7 +6557,7 @@
       <c r="M256" s="16"/>
       <c r="N256" s="17"/>
     </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A257" s="13"/>
       <c r="B257" s="14"/>
       <c r="C257" s="14"/>
@@ -6537,7 +6579,7 @@
       <c r="M257" s="16"/>
       <c r="N257" s="17"/>
     </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A258" s="13"/>
       <c r="B258" s="14"/>
       <c r="C258" s="14"/>
@@ -6559,7 +6601,7 @@
       <c r="M258" s="16"/>
       <c r="N258" s="17"/>
     </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A259" s="13"/>
       <c r="B259" s="14"/>
       <c r="C259" s="14"/>
@@ -6581,7 +6623,7 @@
       <c r="M259" s="16"/>
       <c r="N259" s="17"/>
     </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A260" s="13"/>
       <c r="B260" s="14"/>
       <c r="C260" s="14"/>
@@ -6603,7 +6645,7 @@
       <c r="M260" s="16"/>
       <c r="N260" s="17"/>
     </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A261" s="13"/>
       <c r="B261" s="14"/>
       <c r="C261" s="14"/>
@@ -6625,7 +6667,7 @@
       <c r="M261" s="16"/>
       <c r="N261" s="17"/>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A262" s="13"/>
       <c r="B262" s="14"/>
       <c r="C262" s="14"/>
@@ -6647,7 +6689,7 @@
       <c r="M262" s="16"/>
       <c r="N262" s="17"/>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A263" s="13"/>
       <c r="B263" s="14"/>
       <c r="C263" s="14"/>
@@ -6669,7 +6711,7 @@
       <c r="M263" s="16"/>
       <c r="N263" s="17"/>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A264" s="13"/>
       <c r="B264" s="14"/>
       <c r="C264" s="14"/>
@@ -6691,7 +6733,7 @@
       <c r="M264" s="16"/>
       <c r="N264" s="17"/>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A265" s="13"/>
       <c r="B265" s="14"/>
       <c r="C265" s="14"/>
@@ -6713,7 +6755,7 @@
       <c r="M265" s="16"/>
       <c r="N265" s="17"/>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A266" s="13"/>
       <c r="B266" s="14"/>
       <c r="C266" s="14"/>
@@ -6735,7 +6777,7 @@
       <c r="M266" s="16"/>
       <c r="N266" s="17"/>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A267" s="13"/>
       <c r="B267" s="14"/>
       <c r="C267" s="14"/>
@@ -6757,7 +6799,7 @@
       <c r="M267" s="16"/>
       <c r="N267" s="17"/>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A268" s="13"/>
       <c r="B268" s="14"/>
       <c r="C268" s="14"/>
@@ -6779,7 +6821,7 @@
       <c r="M268" s="16"/>
       <c r="N268" s="17"/>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A269" s="13"/>
       <c r="B269" s="14"/>
       <c r="C269" s="14"/>
@@ -6801,7 +6843,7 @@
       <c r="M269" s="16"/>
       <c r="N269" s="17"/>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A270" s="13"/>
       <c r="B270" s="14"/>
       <c r="C270" s="14"/>
@@ -6823,7 +6865,7 @@
       <c r="M270" s="16"/>
       <c r="N270" s="17"/>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A271" s="13"/>
       <c r="B271" s="14"/>
       <c r="C271" s="14"/>
@@ -6845,7 +6887,7 @@
       <c r="M271" s="16"/>
       <c r="N271" s="17"/>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A272" s="13"/>
       <c r="B272" s="14"/>
       <c r="C272" s="14"/>
@@ -6867,7 +6909,7 @@
       <c r="M272" s="16"/>
       <c r="N272" s="17"/>
     </row>
-    <row r="273" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A273" s="13"/>
       <c r="B273" s="14"/>
       <c r="C273" s="14"/>
@@ -6889,7 +6931,7 @@
       <c r="M273" s="16"/>
       <c r="N273" s="17"/>
     </row>
-    <row r="274" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A274" s="13"/>
       <c r="B274" s="14"/>
       <c r="C274" s="14"/>
@@ -6911,7 +6953,7 @@
       <c r="M274" s="16"/>
       <c r="N274" s="17"/>
     </row>
-    <row r="275" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A275" s="13"/>
       <c r="B275" s="14"/>
       <c r="C275" s="14"/>
@@ -6933,7 +6975,7 @@
       <c r="M275" s="16"/>
       <c r="N275" s="17"/>
     </row>
-    <row r="276" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A276" s="13"/>
       <c r="B276" s="14"/>
       <c r="C276" s="14"/>
@@ -6955,7 +6997,7 @@
       <c r="M276" s="16"/>
       <c r="N276" s="17"/>
     </row>
-    <row r="277" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A277" s="13"/>
       <c r="B277" s="14"/>
       <c r="C277" s="14"/>
@@ -6977,7 +7019,7 @@
       <c r="M277" s="16"/>
       <c r="N277" s="17"/>
     </row>
-    <row r="278" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A278" s="13"/>
       <c r="B278" s="14"/>
       <c r="C278" s="14"/>
@@ -6999,7 +7041,7 @@
       <c r="M278" s="16"/>
       <c r="N278" s="17"/>
     </row>
-    <row r="279" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A279" s="13"/>
       <c r="B279" s="14"/>
       <c r="C279" s="14"/>
@@ -7021,7 +7063,7 @@
       <c r="M279" s="16"/>
       <c r="N279" s="17"/>
     </row>
-    <row r="280" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A280" s="13"/>
       <c r="B280" s="14"/>
       <c r="C280" s="14"/>
@@ -7043,7 +7085,7 @@
       <c r="M280" s="16"/>
       <c r="N280" s="17"/>
     </row>
-    <row r="281" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A281" s="13"/>
       <c r="B281" s="14"/>
       <c r="C281" s="14"/>
@@ -7065,7 +7107,7 @@
       <c r="M281" s="16"/>
       <c r="N281" s="17"/>
     </row>
-    <row r="282" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A282" s="13"/>
       <c r="B282" s="14"/>
       <c r="C282" s="14"/>
@@ -7087,7 +7129,7 @@
       <c r="M282" s="16"/>
       <c r="N282" s="17"/>
     </row>
-    <row r="283" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A283" s="13"/>
       <c r="B283" s="14"/>
       <c r="C283" s="14"/>
@@ -7109,7 +7151,7 @@
       <c r="M283" s="16"/>
       <c r="N283" s="17"/>
     </row>
-    <row r="284" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A284" s="13"/>
       <c r="B284" s="14"/>
       <c r="C284" s="14"/>
@@ -7131,7 +7173,7 @@
       <c r="M284" s="16"/>
       <c r="N284" s="17"/>
     </row>
-    <row r="285" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A285" s="13"/>
       <c r="B285" s="14"/>
       <c r="C285" s="14"/>
@@ -7153,7 +7195,7 @@
       <c r="M285" s="16"/>
       <c r="N285" s="17"/>
     </row>
-    <row r="286" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A286" s="13"/>
       <c r="B286" s="14"/>
       <c r="C286" s="14"/>
@@ -7175,7 +7217,7 @@
       <c r="M286" s="16"/>
       <c r="N286" s="17"/>
     </row>
-    <row r="287" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A287" s="13"/>
       <c r="B287" s="14"/>
       <c r="C287" s="14"/>
@@ -7197,7 +7239,7 @@
       <c r="M287" s="16"/>
       <c r="N287" s="17"/>
     </row>
-    <row r="288" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A288" s="13"/>
       <c r="B288" s="14"/>
       <c r="C288" s="14"/>
@@ -7219,7 +7261,7 @@
       <c r="M288" s="16"/>
       <c r="N288" s="17"/>
     </row>
-    <row r="289" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A289" s="13"/>
       <c r="B289" s="14"/>
       <c r="C289" s="14"/>
@@ -7241,7 +7283,7 @@
       <c r="M289" s="16"/>
       <c r="N289" s="17"/>
     </row>
-    <row r="290" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A290" s="13"/>
       <c r="B290" s="14"/>
       <c r="C290" s="14"/>
@@ -7263,7 +7305,7 @@
       <c r="M290" s="16"/>
       <c r="N290" s="17"/>
     </row>
-    <row r="291" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A291" s="13"/>
       <c r="B291" s="14"/>
       <c r="C291" s="14"/>
@@ -7285,7 +7327,7 @@
       <c r="M291" s="16"/>
       <c r="N291" s="17"/>
     </row>
-    <row r="292" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A292" s="13"/>
       <c r="B292" s="14"/>
       <c r="C292" s="14"/>
@@ -7307,7 +7349,7 @@
       <c r="M292" s="16"/>
       <c r="N292" s="17"/>
     </row>
-    <row r="293" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A293" s="13"/>
       <c r="B293" s="14"/>
       <c r="C293" s="14"/>
@@ -7329,7 +7371,7 @@
       <c r="M293" s="16"/>
       <c r="N293" s="17"/>
     </row>
-    <row r="294" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A294" s="13"/>
       <c r="B294" s="14"/>
       <c r="C294" s="14"/>
@@ -7351,7 +7393,7 @@
       <c r="M294" s="16"/>
       <c r="N294" s="17"/>
     </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A295" s="13"/>
       <c r="B295" s="14"/>
       <c r="C295" s="14"/>
@@ -7373,7 +7415,7 @@
       <c r="M295" s="16"/>
       <c r="N295" s="17"/>
     </row>
-    <row r="296" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A296" s="13"/>
       <c r="B296" s="14"/>
       <c r="C296" s="14"/>
@@ -7395,7 +7437,7 @@
       <c r="M296" s="16"/>
       <c r="N296" s="17"/>
     </row>
-    <row r="297" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A297" s="13"/>
       <c r="B297" s="14"/>
       <c r="C297" s="14"/>
@@ -7417,7 +7459,7 @@
       <c r="M297" s="16"/>
       <c r="N297" s="17"/>
     </row>
-    <row r="298" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A298" s="13"/>
       <c r="B298" s="14"/>
       <c r="C298" s="14"/>
@@ -7439,7 +7481,7 @@
       <c r="M298" s="16"/>
       <c r="N298" s="17"/>
     </row>
-    <row r="299" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A299" s="13"/>
       <c r="B299" s="14"/>
       <c r="C299" s="14"/>
@@ -7461,7 +7503,7 @@
       <c r="M299" s="16"/>
       <c r="N299" s="17"/>
     </row>
-    <row r="300" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A300" s="13"/>
       <c r="B300" s="14"/>
       <c r="C300" s="14"/>
@@ -7483,7 +7525,7 @@
       <c r="M300" s="16"/>
       <c r="N300" s="17"/>
     </row>
-    <row r="301" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A301" s="13"/>
       <c r="B301" s="14"/>
       <c r="C301" s="14"/>
@@ -7505,7 +7547,7 @@
       <c r="M301" s="16"/>
       <c r="N301" s="17"/>
     </row>
-    <row r="302" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A302" s="13"/>
       <c r="B302" s="14"/>
       <c r="C302" s="14"/>
@@ -7527,7 +7569,7 @@
       <c r="M302" s="16"/>
       <c r="N302" s="17"/>
     </row>
-    <row r="303" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A303" s="13"/>
       <c r="B303" s="14"/>
       <c r="C303" s="14"/>
@@ -7549,7 +7591,7 @@
       <c r="M303" s="16"/>
       <c r="N303" s="17"/>
     </row>
-    <row r="304" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A304" s="13"/>
       <c r="B304" s="14"/>
       <c r="C304" s="14"/>
@@ -7571,7 +7613,7 @@
       <c r="M304" s="16"/>
       <c r="N304" s="17"/>
     </row>
-    <row r="305" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A305" s="13"/>
       <c r="B305" s="14"/>
       <c r="C305" s="14"/>
@@ -7593,7 +7635,7 @@
       <c r="M305" s="16"/>
       <c r="N305" s="17"/>
     </row>
-    <row r="306" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A306" s="13"/>
       <c r="B306" s="14"/>
       <c r="C306" s="14"/>
@@ -7615,7 +7657,7 @@
       <c r="M306" s="16"/>
       <c r="N306" s="17"/>
     </row>
-    <row r="307" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A307" s="13"/>
       <c r="B307" s="14"/>
       <c r="C307" s="14"/>
@@ -7637,7 +7679,7 @@
       <c r="M307" s="16"/>
       <c r="N307" s="17"/>
     </row>
-    <row r="308" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A308" s="13"/>
       <c r="B308" s="14"/>
       <c r="C308" s="14"/>
@@ -7659,7 +7701,7 @@
       <c r="M308" s="16"/>
       <c r="N308" s="17"/>
     </row>
-    <row r="309" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A309" s="13"/>
       <c r="B309" s="14"/>
       <c r="C309" s="14"/>
@@ -7681,7 +7723,7 @@
       <c r="M309" s="16"/>
       <c r="N309" s="17"/>
     </row>
-    <row r="310" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A310" s="13"/>
       <c r="B310" s="14"/>
       <c r="C310" s="14"/>
@@ -7703,7 +7745,7 @@
       <c r="M310" s="16"/>
       <c r="N310" s="17"/>
     </row>
-    <row r="311" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A311" s="13"/>
       <c r="B311" s="14"/>
       <c r="C311" s="14"/>
@@ -7725,7 +7767,7 @@
       <c r="M311" s="16"/>
       <c r="N311" s="17"/>
     </row>
-    <row r="312" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A312" s="13"/>
       <c r="B312" s="14"/>
       <c r="C312" s="14"/>
@@ -7747,7 +7789,7 @@
       <c r="M312" s="16"/>
       <c r="N312" s="17"/>
     </row>
-    <row r="313" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A313" s="13"/>
       <c r="B313" s="14"/>
       <c r="C313" s="14"/>
@@ -7769,7 +7811,7 @@
       <c r="M313" s="16"/>
       <c r="N313" s="17"/>
     </row>
-    <row r="314" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A314" s="13"/>
       <c r="B314" s="14"/>
       <c r="C314" s="14"/>
@@ -7791,7 +7833,7 @@
       <c r="M314" s="16"/>
       <c r="N314" s="17"/>
     </row>
-    <row r="315" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A315" s="13"/>
       <c r="B315" s="14"/>
       <c r="C315" s="14"/>
@@ -7813,7 +7855,7 @@
       <c r="M315" s="16"/>
       <c r="N315" s="17"/>
     </row>
-    <row r="316" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A316" s="13"/>
       <c r="B316" s="14"/>
       <c r="C316" s="14"/>
@@ -7835,7 +7877,7 @@
       <c r="M316" s="16"/>
       <c r="N316" s="17"/>
     </row>
-    <row r="317" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A317" s="13"/>
       <c r="B317" s="14"/>
       <c r="C317" s="14"/>
@@ -7857,7 +7899,7 @@
       <c r="M317" s="16"/>
       <c r="N317" s="17"/>
     </row>
-    <row r="318" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A318" s="13"/>
       <c r="B318" s="14"/>
       <c r="C318" s="14"/>
@@ -7879,7 +7921,7 @@
       <c r="M318" s="16"/>
       <c r="N318" s="17"/>
     </row>
-    <row r="319" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A319" s="13"/>
       <c r="B319" s="14"/>
       <c r="C319" s="14"/>
@@ -7901,7 +7943,7 @@
       <c r="M319" s="16"/>
       <c r="N319" s="17"/>
     </row>
-    <row r="320" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A320" s="13"/>
       <c r="B320" s="14"/>
       <c r="C320" s="14"/>
@@ -7923,7 +7965,7 @@
       <c r="M320" s="16"/>
       <c r="N320" s="17"/>
     </row>
-    <row r="321" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A321" s="13"/>
       <c r="B321" s="14"/>
       <c r="C321" s="14"/>
@@ -7945,7 +7987,7 @@
       <c r="M321" s="16"/>
       <c r="N321" s="17"/>
     </row>
-    <row r="322" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A322" s="13"/>
       <c r="B322" s="14"/>
       <c r="C322" s="14"/>
@@ -7967,7 +8009,7 @@
       <c r="M322" s="16"/>
       <c r="N322" s="17"/>
     </row>
-    <row r="323" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A323" s="13"/>
       <c r="B323" s="14"/>
       <c r="C323" s="14"/>
@@ -7989,7 +8031,7 @@
       <c r="M323" s="16"/>
       <c r="N323" s="17"/>
     </row>
-    <row r="324" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A324" s="13"/>
       <c r="B324" s="14"/>
       <c r="C324" s="14"/>
@@ -8011,7 +8053,7 @@
       <c r="M324" s="16"/>
       <c r="N324" s="17"/>
     </row>
-    <row r="325" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A325" s="13"/>
       <c r="B325" s="14"/>
       <c r="C325" s="14"/>
@@ -8033,7 +8075,7 @@
       <c r="M325" s="16"/>
       <c r="N325" s="17"/>
     </row>
-    <row r="326" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A326" s="13"/>
       <c r="B326" s="14"/>
       <c r="C326" s="14"/>
@@ -8055,7 +8097,7 @@
       <c r="M326" s="16"/>
       <c r="N326" s="17"/>
     </row>
-    <row r="327" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A327" s="13"/>
       <c r="B327" s="14"/>
       <c r="C327" s="14"/>
@@ -8077,7 +8119,7 @@
       <c r="M327" s="16"/>
       <c r="N327" s="17"/>
     </row>
-    <row r="328" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A328" s="13"/>
       <c r="B328" s="14"/>
       <c r="C328" s="14"/>
@@ -8099,7 +8141,7 @@
       <c r="M328" s="16"/>
       <c r="N328" s="17"/>
     </row>
-    <row r="329" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A329" s="13"/>
       <c r="B329" s="14"/>
       <c r="C329" s="14"/>
@@ -8121,7 +8163,7 @@
       <c r="M329" s="16"/>
       <c r="N329" s="17"/>
     </row>
-    <row r="330" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A330" s="13"/>
       <c r="B330" s="14"/>
       <c r="C330" s="14"/>
@@ -8143,7 +8185,7 @@
       <c r="M330" s="16"/>
       <c r="N330" s="17"/>
     </row>
-    <row r="331" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A331" s="13"/>
       <c r="B331" s="14"/>
       <c r="C331" s="14"/>
@@ -8165,7 +8207,7 @@
       <c r="M331" s="16"/>
       <c r="N331" s="17"/>
     </row>
-    <row r="332" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A332" s="13"/>
       <c r="B332" s="14"/>
       <c r="C332" s="14"/>
@@ -8187,7 +8229,7 @@
       <c r="M332" s="16"/>
       <c r="N332" s="17"/>
     </row>
-    <row r="333" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A333" s="13"/>
       <c r="B333" s="14"/>
       <c r="C333" s="14"/>
@@ -8209,7 +8251,7 @@
       <c r="M333" s="16"/>
       <c r="N333" s="17"/>
     </row>
-    <row r="334" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A334" s="13"/>
       <c r="B334" s="14"/>
       <c r="C334" s="14"/>
@@ -8231,7 +8273,7 @@
       <c r="M334" s="16"/>
       <c r="N334" s="17"/>
     </row>
-    <row r="335" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A335" s="13"/>
       <c r="B335" s="14"/>
       <c r="C335" s="14"/>
@@ -8253,7 +8295,7 @@
       <c r="M335" s="16"/>
       <c r="N335" s="17"/>
     </row>
-    <row r="336" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A336" s="13"/>
       <c r="B336" s="14"/>
       <c r="C336" s="14"/>
@@ -8275,7 +8317,7 @@
       <c r="M336" s="16"/>
       <c r="N336" s="17"/>
     </row>
-    <row r="337" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A337" s="13"/>
       <c r="B337" s="14"/>
       <c r="C337" s="14"/>
@@ -8297,7 +8339,7 @@
       <c r="M337" s="16"/>
       <c r="N337" s="17"/>
     </row>
-    <row r="338" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A338" s="13"/>
       <c r="B338" s="14"/>
       <c r="C338" s="14"/>
@@ -8319,7 +8361,7 @@
       <c r="M338" s="16"/>
       <c r="N338" s="17"/>
     </row>
-    <row r="339" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A339" s="13"/>
       <c r="B339" s="14"/>
       <c r="C339" s="14"/>
@@ -8341,7 +8383,7 @@
       <c r="M339" s="16"/>
       <c r="N339" s="17"/>
     </row>
-    <row r="340" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A340" s="13"/>
       <c r="B340" s="14"/>
       <c r="C340" s="14"/>
@@ -8363,7 +8405,7 @@
       <c r="M340" s="16"/>
       <c r="N340" s="17"/>
     </row>
-    <row r="341" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A341" s="13"/>
       <c r="B341" s="14"/>
       <c r="C341" s="14"/>
@@ -8385,7 +8427,7 @@
       <c r="M341" s="16"/>
       <c r="N341" s="17"/>
     </row>
-    <row r="342" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A342" s="13"/>
       <c r="B342" s="14"/>
       <c r="C342" s="14"/>
@@ -8407,7 +8449,7 @@
       <c r="M342" s="16"/>
       <c r="N342" s="17"/>
     </row>
-    <row r="343" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A343" s="13"/>
       <c r="B343" s="14"/>
       <c r="C343" s="14"/>
@@ -8429,7 +8471,7 @@
       <c r="M343" s="16"/>
       <c r="N343" s="17"/>
     </row>
-    <row r="344" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A344" s="13"/>
       <c r="B344" s="14"/>
       <c r="C344" s="14"/>
@@ -8451,7 +8493,7 @@
       <c r="M344" s="16"/>
       <c r="N344" s="17"/>
     </row>
-    <row r="345" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A345" s="13"/>
       <c r="B345" s="14"/>
       <c r="C345" s="14"/>
@@ -8473,7 +8515,7 @@
       <c r="M345" s="16"/>
       <c r="N345" s="17"/>
     </row>
-    <row r="346" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A346" s="13"/>
       <c r="B346" s="14"/>
       <c r="C346" s="14"/>
@@ -8495,7 +8537,7 @@
       <c r="M346" s="16"/>
       <c r="N346" s="17"/>
     </row>
-    <row r="347" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A347" s="13"/>
       <c r="B347" s="14"/>
       <c r="C347" s="14"/>
@@ -8517,7 +8559,7 @@
       <c r="M347" s="16"/>
       <c r="N347" s="17"/>
     </row>
-    <row r="348" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A348" s="13"/>
       <c r="B348" s="14"/>
       <c r="C348" s="14"/>
@@ -8539,7 +8581,7 @@
       <c r="M348" s="16"/>
       <c r="N348" s="17"/>
     </row>
-    <row r="349" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A349" s="13"/>
       <c r="B349" s="14"/>
       <c r="C349" s="14"/>
@@ -8561,7 +8603,7 @@
       <c r="M349" s="16"/>
       <c r="N349" s="17"/>
     </row>
-    <row r="350" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A350" s="13"/>
       <c r="B350" s="14"/>
       <c r="C350" s="14"/>
@@ -8583,7 +8625,7 @@
       <c r="M350" s="16"/>
       <c r="N350" s="17"/>
     </row>
-    <row r="351" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A351" s="13"/>
       <c r="B351" s="14"/>
       <c r="C351" s="14"/>
@@ -8605,7 +8647,7 @@
       <c r="M351" s="16"/>
       <c r="N351" s="17"/>
     </row>
-    <row r="352" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A352" s="13"/>
       <c r="B352" s="14"/>
       <c r="C352" s="14"/>
@@ -8627,7 +8669,7 @@
       <c r="M352" s="16"/>
       <c r="N352" s="17"/>
     </row>
-    <row r="353" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A353" s="13"/>
       <c r="B353" s="14"/>
       <c r="C353" s="14"/>
@@ -8649,7 +8691,7 @@
       <c r="M353" s="16"/>
       <c r="N353" s="17"/>
     </row>
-    <row r="354" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A354" s="13"/>
       <c r="B354" s="14"/>
       <c r="C354" s="14"/>
@@ -8671,7 +8713,7 @@
       <c r="M354" s="16"/>
       <c r="N354" s="17"/>
     </row>
-    <row r="355" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A355" s="13"/>
       <c r="B355" s="14"/>
       <c r="C355" s="14"/>
@@ -8693,7 +8735,7 @@
       <c r="M355" s="16"/>
       <c r="N355" s="17"/>
     </row>
-    <row r="356" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A356" s="13"/>
       <c r="B356" s="14"/>
       <c r="C356" s="14"/>
@@ -8715,7 +8757,7 @@
       <c r="M356" s="16"/>
       <c r="N356" s="17"/>
     </row>
-    <row r="357" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A357" s="13"/>
       <c r="B357" s="14"/>
       <c r="C357" s="14"/>
@@ -8737,7 +8779,7 @@
       <c r="M357" s="16"/>
       <c r="N357" s="17"/>
     </row>
-    <row r="358" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A358" s="13"/>
       <c r="B358" s="14"/>
       <c r="C358" s="14"/>
@@ -8759,7 +8801,7 @@
       <c r="M358" s="16"/>
       <c r="N358" s="17"/>
     </row>
-    <row r="359" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A359" s="13"/>
       <c r="B359" s="14"/>
       <c r="C359" s="14"/>
@@ -8781,7 +8823,7 @@
       <c r="M359" s="16"/>
       <c r="N359" s="17"/>
     </row>
-    <row r="360" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A360" s="13"/>
       <c r="B360" s="14"/>
       <c r="C360" s="14"/>
@@ -8803,7 +8845,7 @@
       <c r="M360" s="16"/>
       <c r="N360" s="17"/>
     </row>
-    <row r="361" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A361" s="13"/>
       <c r="B361" s="14"/>
       <c r="C361" s="14"/>
@@ -8825,7 +8867,7 @@
       <c r="M361" s="16"/>
       <c r="N361" s="17"/>
     </row>
-    <row r="362" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A362" s="13"/>
       <c r="B362" s="14"/>
       <c r="C362" s="14"/>
@@ -8847,7 +8889,7 @@
       <c r="M362" s="16"/>
       <c r="N362" s="17"/>
     </row>
-    <row r="363" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A363" s="13"/>
       <c r="B363" s="14"/>
       <c r="C363" s="14"/>
@@ -8869,7 +8911,7 @@
       <c r="M363" s="16"/>
       <c r="N363" s="17"/>
     </row>
-    <row r="364" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A364" s="13"/>
       <c r="B364" s="14"/>
       <c r="C364" s="14"/>
@@ -8891,7 +8933,7 @@
       <c r="M364" s="16"/>
       <c r="N364" s="17"/>
     </row>
-    <row r="365" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A365" s="13"/>
       <c r="B365" s="14"/>
       <c r="C365" s="14"/>
@@ -8913,7 +8955,7 @@
       <c r="M365" s="16"/>
       <c r="N365" s="17"/>
     </row>
-    <row r="366" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A366" s="13"/>
       <c r="B366" s="14"/>
       <c r="C366" s="14"/>
@@ -8935,7 +8977,7 @@
       <c r="M366" s="16"/>
       <c r="N366" s="17"/>
     </row>
-    <row r="367" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A367" s="13"/>
       <c r="B367" s="14"/>
       <c r="C367" s="14"/>
@@ -8957,7 +8999,7 @@
       <c r="M367" s="16"/>
       <c r="N367" s="17"/>
     </row>
-    <row r="368" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A368" s="13"/>
       <c r="B368" s="14"/>
       <c r="C368" s="14"/>
@@ -8979,7 +9021,7 @@
       <c r="M368" s="16"/>
       <c r="N368" s="17"/>
     </row>
-    <row r="369" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A369" s="13"/>
       <c r="B369" s="14"/>
       <c r="C369" s="14"/>
@@ -9001,7 +9043,7 @@
       <c r="M369" s="16"/>
       <c r="N369" s="17"/>
     </row>
-    <row r="370" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A370" s="13"/>
       <c r="B370" s="14"/>
       <c r="C370" s="14"/>
@@ -9023,7 +9065,7 @@
       <c r="M370" s="16"/>
       <c r="N370" s="17"/>
     </row>
-    <row r="371" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A371" s="13"/>
       <c r="B371" s="14"/>
       <c r="C371" s="14"/>
@@ -9045,7 +9087,7 @@
       <c r="M371" s="16"/>
       <c r="N371" s="17"/>
     </row>
-    <row r="372" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A372" s="13"/>
       <c r="B372" s="14"/>
       <c r="C372" s="14"/>
@@ -9067,7 +9109,7 @@
       <c r="M372" s="16"/>
       <c r="N372" s="17"/>
     </row>
-    <row r="373" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A373" s="13"/>
       <c r="B373" s="14"/>
       <c r="C373" s="14"/>
@@ -9089,7 +9131,7 @@
       <c r="M373" s="16"/>
       <c r="N373" s="17"/>
     </row>
-    <row r="374" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A374" s="13"/>
       <c r="B374" s="14"/>
       <c r="C374" s="14"/>
@@ -9111,7 +9153,7 @@
       <c r="M374" s="16"/>
       <c r="N374" s="17"/>
     </row>
-    <row r="375" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A375" s="13"/>
       <c r="B375" s="14"/>
       <c r="C375" s="14"/>
@@ -9133,7 +9175,7 @@
       <c r="M375" s="16"/>
       <c r="N375" s="17"/>
     </row>
-    <row r="376" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A376" s="13"/>
       <c r="B376" s="14"/>
       <c r="C376" s="14"/>
@@ -9155,7 +9197,7 @@
       <c r="M376" s="16"/>
       <c r="N376" s="17"/>
     </row>
-    <row r="377" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A377" s="13"/>
       <c r="B377" s="14"/>
       <c r="C377" s="14"/>
@@ -9177,7 +9219,7 @@
       <c r="M377" s="16"/>
       <c r="N377" s="17"/>
     </row>
-    <row r="378" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A378" s="13"/>
       <c r="B378" s="14"/>
       <c r="C378" s="14"/>
@@ -9199,7 +9241,7 @@
       <c r="M378" s="16"/>
       <c r="N378" s="17"/>
     </row>
-    <row r="379" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A379" s="13"/>
       <c r="B379" s="14"/>
       <c r="C379" s="14"/>
@@ -9221,7 +9263,7 @@
       <c r="M379" s="16"/>
       <c r="N379" s="17"/>
     </row>
-    <row r="380" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A380" s="13"/>
       <c r="B380" s="14"/>
       <c r="C380" s="14"/>
@@ -9243,7 +9285,7 @@
       <c r="M380" s="16"/>
       <c r="N380" s="17"/>
     </row>
-    <row r="381" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A381" s="13"/>
       <c r="B381" s="14"/>
       <c r="C381" s="14"/>
@@ -9265,7 +9307,7 @@
       <c r="M381" s="16"/>
       <c r="N381" s="17"/>
     </row>
-    <row r="382" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A382" s="13"/>
       <c r="B382" s="14"/>
       <c r="C382" s="14"/>
@@ -9287,7 +9329,7 @@
       <c r="M382" s="16"/>
       <c r="N382" s="17"/>
     </row>
-    <row r="383" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A383" s="13"/>
       <c r="B383" s="14"/>
       <c r="C383" s="14"/>
@@ -9309,7 +9351,7 @@
       <c r="M383" s="16"/>
       <c r="N383" s="17"/>
     </row>
-    <row r="384" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A384" s="13"/>
       <c r="B384" s="14"/>
       <c r="C384" s="14"/>
@@ -9331,7 +9373,7 @@
       <c r="M384" s="16"/>
       <c r="N384" s="17"/>
     </row>
-    <row r="385" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A385" s="13"/>
       <c r="B385" s="14"/>
       <c r="C385" s="14"/>
@@ -9353,7 +9395,7 @@
       <c r="M385" s="16"/>
       <c r="N385" s="17"/>
     </row>
-    <row r="386" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A386" s="13"/>
       <c r="B386" s="14"/>
       <c r="C386" s="14"/>
@@ -9375,7 +9417,7 @@
       <c r="M386" s="16"/>
       <c r="N386" s="17"/>
     </row>
-    <row r="387" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A387" s="13"/>
       <c r="B387" s="14"/>
       <c r="C387" s="14"/>
@@ -9397,7 +9439,7 @@
       <c r="M387" s="16"/>
       <c r="N387" s="17"/>
     </row>
-    <row r="388" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A388" s="13"/>
       <c r="B388" s="14"/>
       <c r="C388" s="14"/>
@@ -9419,7 +9461,7 @@
       <c r="M388" s="16"/>
       <c r="N388" s="17"/>
     </row>
-    <row r="389" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A389" s="13"/>
       <c r="B389" s="14"/>
       <c r="C389" s="14"/>
@@ -9441,7 +9483,7 @@
       <c r="M389" s="16"/>
       <c r="N389" s="17"/>
     </row>
-    <row r="390" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A390" s="13"/>
       <c r="B390" s="14"/>
       <c r="C390" s="14"/>
@@ -9463,7 +9505,7 @@
       <c r="M390" s="16"/>
       <c r="N390" s="17"/>
     </row>
-    <row r="391" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A391" s="13"/>
       <c r="B391" s="14"/>
       <c r="C391" s="14"/>
@@ -9485,7 +9527,7 @@
       <c r="M391" s="16"/>
       <c r="N391" s="17"/>
     </row>
-    <row r="392" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A392" s="13"/>
       <c r="B392" s="14"/>
       <c r="C392" s="14"/>
@@ -9507,7 +9549,7 @@
       <c r="M392" s="16"/>
       <c r="N392" s="17"/>
     </row>
-    <row r="393" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A393" s="13"/>
       <c r="B393" s="14"/>
       <c r="C393" s="14"/>
@@ -9529,7 +9571,7 @@
       <c r="M393" s="16"/>
       <c r="N393" s="17"/>
     </row>
-    <row r="394" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A394" s="13"/>
       <c r="B394" s="14"/>
       <c r="C394" s="14"/>
@@ -9551,7 +9593,7 @@
       <c r="M394" s="16"/>
       <c r="N394" s="17"/>
     </row>
-    <row r="395" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A395" s="13"/>
       <c r="B395" s="14"/>
       <c r="C395" s="14"/>
@@ -9573,7 +9615,7 @@
       <c r="M395" s="16"/>
       <c r="N395" s="17"/>
     </row>
-    <row r="396" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A396" s="13"/>
       <c r="B396" s="14"/>
       <c r="C396" s="14"/>
@@ -9595,7 +9637,7 @@
       <c r="M396" s="16"/>
       <c r="N396" s="17"/>
     </row>
-    <row r="397" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A397" s="13"/>
       <c r="B397" s="14"/>
       <c r="C397" s="14"/>
@@ -9617,7 +9659,7 @@
       <c r="M397" s="16"/>
       <c r="N397" s="17"/>
     </row>
-    <row r="398" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A398" s="13"/>
       <c r="B398" s="14"/>
       <c r="C398" s="14"/>
@@ -9639,7 +9681,7 @@
       <c r="M398" s="16"/>
       <c r="N398" s="17"/>
     </row>
-    <row r="399" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A399" s="13"/>
       <c r="B399" s="14"/>
       <c r="C399" s="14"/>
@@ -9661,7 +9703,7 @@
       <c r="M399" s="16"/>
       <c r="N399" s="17"/>
     </row>
-    <row r="400" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A400" s="13"/>
       <c r="B400" s="14"/>
       <c r="C400" s="14"/>
@@ -9683,7 +9725,7 @@
       <c r="M400" s="16"/>
       <c r="N400" s="17"/>
     </row>
-    <row r="401" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A401" s="13"/>
       <c r="B401" s="14"/>
       <c r="C401" s="14"/>

</xml_diff>